<commit_message>
Baseline version: warehouse simulation sheets completed
</commit_message>
<xml_diff>
--- a/Warehouse_Operations_Simulation.xlsx
+++ b/Warehouse_Operations_Simulation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Upgrade skill\1. Excel - Data Analytics\Project\Warehouse Operations Portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7AEE89B-4558-4D5B-BC50-C5B24B15010F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{101C287A-8C0B-4552-8526-2818462A53FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" tabRatio="500" firstSheet="9" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_Master_Material" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Add cycle count worksheet
</commit_message>
<xml_diff>
--- a/Warehouse_Operations_Simulation.xlsx
+++ b/Warehouse_Operations_Simulation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Upgrade skill\1. Excel - Data Analytics\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C643BF5E-8E1F-4ADF-874B-F23B752043BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{700275E2-3C0F-4E86-A8FD-1C0B2EE12777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2063,7 +2063,93 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="199">
+  <dxfs count="203">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFB7B7B7"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFB7B7B7"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFB7B7B7"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFB7B7B7"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FFB7B7B7"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFB7B7B7"/>
+        </right>
+        <top style="thin">
+          <color rgb="FFB7B7B7"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FFB7B7B7"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <i/>
@@ -5251,21 +5337,21 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="tbl_MasterMaterial" displayName="tbl_MasterMaterial" ref="A3:O23" totalsRowShown="0">
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Material Code" dataDxfId="198"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Material Description" dataDxfId="197"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Material Group" dataDxfId="196"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Material Code" dataDxfId="202"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Material Description" dataDxfId="201"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Material Group" dataDxfId="200"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Base UoM"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Primary Supplier Code"/>
-    <tableColumn id="24" xr3:uid="{0F116849-4911-4B80-B390-3C1C1D0A9D49}" name="Default Storage Location" dataDxfId="195"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Standard Cost (per Base UoM)" dataDxfId="194"/>
-    <tableColumn id="5" xr3:uid="{01500A3B-77EE-4BAE-BC67-664F09E22186}" name="ABC Classification" dataDxfId="193"/>
+    <tableColumn id="24" xr3:uid="{0F116849-4911-4B80-B390-3C1C1D0A9D49}" name="Default Storage Location" dataDxfId="199"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Standard Cost (per Base UoM)" dataDxfId="198"/>
+    <tableColumn id="5" xr3:uid="{01500A3B-77EE-4BAE-BC67-664F09E22186}" name="ABC Classification" dataDxfId="197"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Criticality Flag"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Storage/Handling Class"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Min Stock Level"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Max Stock Level"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Min Stock Level" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Max Stock Level" dataDxfId="0"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Lead Time (Days)"/>
     <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Status"/>
-    <tableColumn id="22" xr3:uid="{BC7C3BEF-CB66-4A5F-9E71-E29F8E60C070}" name="Remarks" dataDxfId="192"/>
+    <tableColumn id="22" xr3:uid="{BC7C3BEF-CB66-4A5F-9E71-E29F8E60C070}" name="Remarks" dataDxfId="196"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5279,36 +5365,36 @@
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="Count Line"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="Count Date"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0A00-000004000000}" name="Material Code"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0A00-000005000000}" name="Material Description" dataDxfId="96">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0A00-000005000000}" name="Material Description" dataDxfId="100">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_CycleCount[[#This Row],[Material Code]],tbl_MasterMaterial[Material Code],tbl_MasterMaterial[Material Description])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="20" xr3:uid="{42D72B1C-0469-448F-89C5-AE97F1EFA4A3}" name="ABC Classification" dataDxfId="95">
+    <tableColumn id="20" xr3:uid="{42D72B1C-0469-448F-89C5-AE97F1EFA4A3}" name="ABC Classification" dataDxfId="99">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_CycleCount[[#This Row],[Material Code]],tbl_MasterMaterial[Material Code],tbl_MasterMaterial[ABC Classification])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0A00-000008000000}" name="Count Location (Ref)" dataDxfId="94"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0A00-000009000000}" name="System Qty (Ref)" dataDxfId="93">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0A00-000008000000}" name="Count Location (Ref)" dataDxfId="98"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0A00-000009000000}" name="System Qty (Ref)" dataDxfId="97">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_CycleCount[[#This Row],[Material Code]],'10_Stock_Card'!F4:F32,'10_Stock_Card'!M4:M32,"",,-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0A00-00000A000000}" name="Physical Count" dataDxfId="92"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0A00-00000B000000}" name="Variance (Qty)" dataDxfId="91">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0A00-00000A000000}" name="Physical Count" dataDxfId="96"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0A00-00000B000000}" name="Variance (Qty)" dataDxfId="95">
       <calculatedColumnFormula>tbl_CycleCount[[#This Row],[Physical Count]]-tbl_CycleCount[[#This Row],[System Qty (Ref)]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0A00-00000C000000}" name="Variance %" dataDxfId="90">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0A00-00000C000000}" name="Variance %" dataDxfId="94">
       <calculatedColumnFormula>IFERROR(tbl_CycleCount[[#This Row],[Variance (Qty)]]/tbl_CycleCount[[#This Row],[System Qty (Ref)]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0A00-00000D000000}" name="Unit Cost (Ref)" dataDxfId="89">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0A00-00000D000000}" name="Unit Cost (Ref)" dataDxfId="93">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_CycleCount[[#This Row],[Material Code]],tbl_MasterMaterial[Material Code],tbl_MasterMaterial[Standard Cost (per Base UoM)])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0A00-00000E000000}" name="Variance Value" dataDxfId="88">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0A00-00000E000000}" name="Variance Value" dataDxfId="92">
       <calculatedColumnFormula>tbl_CycleCount[[#This Row],[Variance (Qty)]]*tbl_CycleCount[[#This Row],[Unit Cost (Ref)]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0A00-00000F000000}" name="Count Result" dataDxfId="87"/>
-    <tableColumn id="7" xr3:uid="{19FA728F-5901-4A45-82C7-A24BD8CD672D}" name="Count By" dataDxfId="86"/>
-    <tableColumn id="6" xr3:uid="{40535110-8F23-4B6C-8557-AF648D9A2B41}" name="Verified By" dataDxfId="85"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0A00-000010000000}" name="Root Cause" dataDxfId="84"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0A00-00000F000000}" name="Count Result" dataDxfId="91"/>
+    <tableColumn id="7" xr3:uid="{19FA728F-5901-4A45-82C7-A24BD8CD672D}" name="Count By" dataDxfId="90"/>
+    <tableColumn id="6" xr3:uid="{40535110-8F23-4B6C-8557-AF648D9A2B41}" name="Verified By" dataDxfId="89"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0A00-000010000000}" name="Root Cause" dataDxfId="88"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0A00-000011000000}" name="Adjustment Status"/>
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0A00-000012000000}" name="Remarks"/>
-    <tableColumn id="19" xr3:uid="{2718145A-3CE3-42EB-A2A9-5B850CE78E6D}" name="Count Line Key (Helper)" dataDxfId="83">
+    <tableColumn id="19" xr3:uid="{2718145A-3CE3-42EB-A2A9-5B850CE78E6D}" name="Count Line Key (Helper)" dataDxfId="87">
       <calculatedColumnFormula>tbl_CycleCount[[#This Row],[Count Number]]&amp;"-"&amp;tbl_CycleCount[[#This Row],[Count Line]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5341,7 +5427,7 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Location Code"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Location Description"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Zone"/>
-    <tableColumn id="8" xr3:uid="{276A2345-C837-4FC6-B4E0-FF35EB523268}" name="Location Type" dataDxfId="191"/>
+    <tableColumn id="8" xr3:uid="{276A2345-C837-4FC6-B4E0-FF35EB523268}" name="Location Type" dataDxfId="195"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Storage/Handling Requirement"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Pickable Flag"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Capacity (Max Qty)"/>
@@ -5362,37 +5448,37 @@
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="PO Line"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="PO Date"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="Supplier Code"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Supplier Name" dataDxfId="190">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="Supplier Name" dataDxfId="194">
       <calculatedColumnFormula>VLOOKUP(tbl_PurchaseOrder[[#This Row],[Supplier Code]],tbl_MasterSupplier[],2,FALSE)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0300-000006000000}" name="Material Code"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="Material Description" dataDxfId="189">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0300-000007000000}" name="Material Description" dataDxfId="193">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PurchaseOrder[[#This Row],[Material Code]],tbl_MasterMaterial[Material Code],tbl_MasterMaterial[Material Description])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="Purchase UoM" dataDxfId="188"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="Ordered Qty" dataDxfId="187" totalsRowDxfId="186"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="Unit Price" dataDxfId="185" totalsRowDxfId="184"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="Line Total" dataDxfId="183" totalsRowDxfId="182">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0300-000008000000}" name="Purchase UoM" dataDxfId="192"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0300-000009000000}" name="Ordered Qty" dataDxfId="191" totalsRowDxfId="190"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0300-00000A000000}" name="Unit Price" dataDxfId="189" totalsRowDxfId="188"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0300-00000B000000}" name="Line Total" dataDxfId="187" totalsRowDxfId="186">
       <calculatedColumnFormula>tbl_PurchaseOrder[[#This Row],[Ordered Qty]]*J4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0300-000010000000}" name="Order Priority" dataDxfId="181" totalsRowDxfId="180"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0300-000010000000}" name="Order Priority" dataDxfId="185" totalsRowDxfId="184"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0300-000011000000}" name="Lead Time (Days)">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PurchaseOrder[[#This Row],[Material Code]],tbl_MasterMaterial[Material Code],tbl_MasterMaterial[Lead Time (Days)])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0300-000012000000}" name="Expected Delivery Date" dataDxfId="179">
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0300-000012000000}" name="Expected Delivery Date" dataDxfId="183">
       <calculatedColumnFormula>tbl_PurchaseOrder[[#This Row],[PO Date]]+tbl_PurchaseOrder[[#This Row],[Lead Time (Days)]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{09E53041-1B48-4B81-BCF8-287332AE53AE}" name="Received Qty" dataDxfId="178" totalsRowDxfId="177">
+    <tableColumn id="13" xr3:uid="{09E53041-1B48-4B81-BCF8-287332AE53AE}" name="Received Qty" dataDxfId="182" totalsRowDxfId="181">
       <calculatedColumnFormula>SUMIFS(tbl_GoodsReceipt[Received Qty],tbl_GoodsReceipt[PO Line Key (Helper)],tbl_PurchaseOrder[[#This Row],[PO Line Key (Helper)]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{123695AE-1CB2-4070-BEE2-29FE092ACFA7}" name="Outstanding Qty" dataDxfId="176" totalsRowDxfId="175">
+    <tableColumn id="14" xr3:uid="{123695AE-1CB2-4070-BEE2-29FE092ACFA7}" name="Outstanding Qty" dataDxfId="180" totalsRowDxfId="179">
       <calculatedColumnFormula>IFERROR(tbl_PurchaseOrder[[#This Row],[Received Qty]]-tbl_PurchaseOrder[[#This Row],[Ordered Qty]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0300-000014000000}" name="PO Status" dataDxfId="174">
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0300-000014000000}" name="PO Status" dataDxfId="178">
       <calculatedColumnFormula>IF(tbl_PurchaseOrder[[#This Row],[Received Qty]]=0,"Open",IF(tbl_PurchaseOrder[[#This Row],[Received Qty]]&lt;tbl_PurchaseOrder[[#This Row],[Ordered Qty]],"Partial", "Closed"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0300-000015000000}" name="Remarks" dataDxfId="173"/>
-    <tableColumn id="19" xr3:uid="{195CE6D1-9D3F-4D81-9DE2-B82EEBF35742}" name="PO Line Key (Helper)" dataDxfId="172" totalsRowDxfId="171">
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0300-000015000000}" name="Remarks" dataDxfId="177"/>
+    <tableColumn id="19" xr3:uid="{195CE6D1-9D3F-4D81-9DE2-B82EEBF35742}" name="PO Line Key (Helper)" dataDxfId="176" totalsRowDxfId="175">
       <calculatedColumnFormula>tbl_PurchaseOrder[[#This Row],[PO Number]]&amp;"-"&amp;tbl_PurchaseOrder[[#This Row],[PO Line]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5411,52 +5497,52 @@
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="GR Line"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="GR Date"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0400-000004000000}" name="PO Number"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="PO Line" dataDxfId="170"/>
-    <tableColumn id="29" xr3:uid="{32467FAF-3D7D-4CA5-9707-3FB4E795D1FA}" name="PO Line Key (Helper)" dataDxfId="169">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0400-000005000000}" name="PO Line" dataDxfId="174"/>
+    <tableColumn id="29" xr3:uid="{32467FAF-3D7D-4CA5-9707-3FB4E795D1FA}" name="PO Line Key (Helper)" dataDxfId="173">
       <calculatedColumnFormula>tbl_GoodsReceipt[[#This Row],[PO Number]]&amp;"-"&amp;tbl_GoodsReceipt[[#This Row],[PO Line]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{E8DA1EE4-E020-4801-93F4-A35A7E1B2656}" name="Supplier Code" dataDxfId="168">
+    <tableColumn id="6" xr3:uid="{E8DA1EE4-E020-4801-93F4-A35A7E1B2656}" name="Supplier Code" dataDxfId="172">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_GoodsReceipt[[#This Row],[PO Line Key (Helper)]],tbl_PurchaseOrder[PO Line Key (Helper)],tbl_PurchaseOrder[Supplier Code])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="Supplier Name" dataDxfId="167">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0400-000007000000}" name="Supplier Name" dataDxfId="171">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_GoodsReceipt[[#This Row],[Supplier Code]],tbl_MasterSupplier[Supplier Code],tbl_MasterSupplier[Supplier Name])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="Material Code" dataDxfId="166">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0400-000008000000}" name="Material Code" dataDxfId="170">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_GoodsReceipt[[#This Row],[PO Line Key (Helper)]],tbl_PurchaseOrder[PO Line Key (Helper)],tbl_PurchaseOrder[Material Code])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="Material Description" dataDxfId="165">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0400-000009000000}" name="Material Description" dataDxfId="169">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_GoodsReceipt[[#This Row],[Material Code]],tbl_MasterMaterial[Material Code],tbl_MasterMaterial[Material Description])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0400-00000A000000}" name="Order Qty" dataDxfId="164">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0400-00000A000000}" name="Order Qty" dataDxfId="168">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_GoodsReceipt[[#This Row],[PO Line Key (Helper)]],tbl_PurchaseOrder[PO Line Key (Helper)],tbl_PurchaseOrder[Ordered Qty])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0400-00000C000000}" name="Purchase UoM" dataDxfId="163">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0400-00000C000000}" name="Purchase UoM" dataDxfId="167">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_GoodsReceipt[[#This Row],[PO Line Key (Helper)]],tbl_PurchaseOrder[PO Line Key (Helper)],tbl_PurchaseOrder[Purchase UoM])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0400-00000B000000}" name="Unit Price" dataDxfId="162">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0400-00000B000000}" name="Unit Price" dataDxfId="166">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_GoodsReceipt[[#This Row],[PO Line Key (Helper)]],tbl_PurchaseOrder[PO Line Key (Helper)],tbl_PurchaseOrder[Unit Price])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0400-000014000000}" name="Expected Delivery Date" dataDxfId="161">
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0400-000014000000}" name="Expected Delivery Date" dataDxfId="165">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_GoodsReceipt[[#This Row],[PO Line Key (Helper)]],tbl_PurchaseOrder[PO Line Key (Helper)],tbl_PurchaseOrder[Expected Delivery Date])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{76F9E9A1-1F34-4FAD-9BFD-02A48B886435}" name="Delivery Note No." dataDxfId="160"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0400-000013000000}" name="Receiving Dock" dataDxfId="159"/>
-    <tableColumn id="27" xr3:uid="{C970C051-0950-4A04-BC06-F42CE88CB783}" name="Received By" dataDxfId="158"/>
+    <tableColumn id="21" xr3:uid="{76F9E9A1-1F34-4FAD-9BFD-02A48B886435}" name="Delivery Note No." dataDxfId="164"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0400-000013000000}" name="Receiving Dock" dataDxfId="163"/>
+    <tableColumn id="27" xr3:uid="{C970C051-0950-4A04-BC06-F42CE88CB783}" name="Received By" dataDxfId="162"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0400-00000D000000}" name="Received Qty"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0400-00000E000000}" name="Accepted Qty"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0400-00000F000000}" name="Rejected Qty" dataDxfId="157">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0400-00000F000000}" name="Rejected Qty" dataDxfId="161">
       <calculatedColumnFormula>tbl_GoodsReceipt[[#This Row],[Received Qty]]-tbl_GoodsReceipt[[#This Row],[Accepted Qty]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="16" xr3:uid="{00000000-0010-0000-0400-000010000000}" name="Inspection Result"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0400-000011000000}" name="Rejection Reason"/>
     <tableColumn id="18" xr3:uid="{00000000-0010-0000-0400-000012000000}" name="Batch/Lot Number"/>
-    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0400-000016000000}" name="Received Variance" dataDxfId="156">
+    <tableColumn id="22" xr3:uid="{00000000-0010-0000-0400-000016000000}" name="Received Variance" dataDxfId="160">
       <calculatedColumnFormula>tbl_GoodsReceipt[[#This Row],[Received Qty]]-tbl_GoodsReceipt[[#This Row],[Order Qty]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="23" xr3:uid="{00000000-0010-0000-0400-000017000000}" name="Received Variance %">
       <calculatedColumnFormula>IFERROR(tbl_GoodsReceipt[[#This Row],[Received Variance]]/tbl_GoodsReceipt[[#This Row],[Order Qty]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="28" xr3:uid="{9903FC18-7740-482D-9ABE-94B8CD52CA29}" name="Delivery Status" dataDxfId="155">
+    <tableColumn id="28" xr3:uid="{9903FC18-7740-482D-9ABE-94B8CD52CA29}" name="Delivery Status" dataDxfId="159">
       <calculatedColumnFormula>IF(tbl_GoodsReceipt[[#This Row],[GR Date]]&lt;=tbl_GoodsReceipt[[#This Row],[Expected Delivery Date]],"On-time","Late")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="25" xr3:uid="{00000000-0010-0000-0400-000019000000}" name="Remarks"/>
@@ -5475,50 +5561,50 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="Put Away Number"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="Put Away Line"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0500-000003000000}" name="Put Away Date"/>
-    <tableColumn id="9" xr3:uid="{3D1409EE-9BE5-4C77-8E8C-75FBB533A1BA}" name="GR Date" dataDxfId="154">
+    <tableColumn id="9" xr3:uid="{3D1409EE-9BE5-4C77-8E8C-75FBB533A1BA}" name="GR Date" dataDxfId="158">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PutAway[[#This Row],[GR Line Key (Helper)]],tbl_GoodsReceipt[GR Line Key (Helper)],tbl_GoodsReceipt[GR Date])</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0500-000004000000}" name="GR Number"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="GR Line" dataDxfId="153"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="GR Line Key (Helper)" dataDxfId="152">
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0500-000005000000}" name="GR Line" dataDxfId="157"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0500-000006000000}" name="GR Line Key (Helper)" dataDxfId="156">
       <calculatedColumnFormula>tbl_PutAway[[#This Row],[GR Number]]&amp;"-"&amp;tbl_PutAway[[#This Row],[GR Line]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0500-000007000000}" name="Material Code">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PutAway[[#This Row],[GR Line Key (Helper)]],tbl_GoodsReceipt[GR Line Key (Helper)],tbl_GoodsReceipt[Material Code])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="Material Description" dataDxfId="151">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0500-000008000000}" name="Material Description" dataDxfId="155">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PutAway[[#This Row],[Material Code]],tbl_GoodsReceipt[Material Code],tbl_GoodsReceipt[Material Description])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{17CC66FF-3B10-4724-A531-9ABD3C5CB8D1}" name="Batch/Lot Number" dataDxfId="150">
+    <tableColumn id="23" xr3:uid="{17CC66FF-3B10-4724-A531-9ABD3C5CB8D1}" name="Batch/Lot Number" dataDxfId="154">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PutAway[[#This Row],[GR Line Key (Helper)]],tbl_GoodsReceipt[GR Line Key (Helper)],tbl_GoodsReceipt[Batch/Lot Number])</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0500-00000C000000}" name="Accepted Qty">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PutAway[[#This Row],[GR Line Key (Helper)]],tbl_GoodsReceipt[GR Line Key (Helper)],tbl_GoodsReceipt[Accepted Qty])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{28CCFCA5-F3BC-430A-80E6-5C20D5AAAE8F}" name="Purchase UoM" dataDxfId="149">
+    <tableColumn id="17" xr3:uid="{28CCFCA5-F3BC-430A-80E6-5C20D5AAAE8F}" name="Purchase UoM" dataDxfId="153">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PutAway[[#This Row],[GR Line Key (Helper)]],tbl_GoodsReceipt[GR Line Key (Helper)],tbl_GoodsReceipt[Purchase UoM])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{0A641E53-0249-44B9-9E19-52E853A7C026}" name="Put Away Qty" dataDxfId="148"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0500-00000D000000}" name="Base UoM" dataDxfId="147">
+    <tableColumn id="16" xr3:uid="{0A641E53-0249-44B9-9E19-52E853A7C026}" name="Put Away Qty" dataDxfId="152"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0500-00000D000000}" name="Base UoM" dataDxfId="151">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PutAway[[#This Row],[Material Code]],tbl_MasterMaterial[Material Code],tbl_MasterMaterial[Base UoM])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0500-00000F000000}" name="From Location" dataDxfId="146">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0500-00000F000000}" name="From Location" dataDxfId="150">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PutAway[[#This Row],[GR Line Key (Helper)]],tbl_GoodsReceipt[GR Line Key (Helper)],tbl_GoodsReceipt[Receiving Dock])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{1E1EA826-7DDD-4C65-AB2E-9676F8A827A7}" name="Suggested Storage Location (Ref)" dataDxfId="145">
+    <tableColumn id="10" xr3:uid="{1E1EA826-7DDD-4C65-AB2E-9676F8A827A7}" name="Suggested Storage Location (Ref)" dataDxfId="149">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PutAway[[#This Row],[Material Code]],tbl_MasterMaterial[Material Code],tbl_MasterMaterial[Default Storage Location])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0500-00000E000000}" name="Storage/Handling Class" dataDxfId="144">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0500-00000E000000}" name="Storage/Handling Class" dataDxfId="148">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PutAway[[#This Row],[Material Code]],tbl_MasterMaterial[Material Code],tbl_MasterMaterial[Storage/Handling Class])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="24" xr3:uid="{BB70C6C7-B755-4415-A577-FB1FBECE67FD}" name="To Location" dataDxfId="143"/>
-    <tableColumn id="19" xr3:uid="{1445C40B-D3A5-4C1B-9654-FF2E02CAEB6A}" name="Location Storage/Handling Requirement" dataDxfId="142">
+    <tableColumn id="24" xr3:uid="{BB70C6C7-B755-4415-A577-FB1FBECE67FD}" name="To Location" dataDxfId="147"/>
+    <tableColumn id="19" xr3:uid="{1445C40B-D3A5-4C1B-9654-FF2E02CAEB6A}" name="Location Storage/Handling Requirement" dataDxfId="146">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PutAway[[#This Row],[To Location]],tbl_MasterLocation[Location Code],tbl_MasterLocation[Storage/Handling Requirement])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="20" xr3:uid="{47D4BE73-8080-42B6-985B-6CB165C06B54}" name="Location Match Check" dataDxfId="141">
+    <tableColumn id="20" xr3:uid="{47D4BE73-8080-42B6-985B-6CB165C06B54}" name="Location Match Check" dataDxfId="145">
       <calculatedColumnFormula>IF(tbl_PutAway[[#This Row],[Location Storage/Handling Requirement]]=tbl_PutAway[[#This Row],[Storage/Handling Class]],"Match","Mismatch - Review")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0500-000012000000}" name="Put Away Status" dataDxfId="140"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0500-000012000000}" name="Put Away Status" dataDxfId="144"/>
     <tableColumn id="21" xr3:uid="{00000000-0010-0000-0500-000015000000}" name="Remarks"/>
     <tableColumn id="22" xr3:uid="{00000000-0010-0000-0500-000016000000}" name="Put-Away Line Key (Helper)">
       <calculatedColumnFormula>tbl_PutAway[[#This Row],[Put Away Number]]&amp;"-"&amp;tbl_PutAway[[#This Row],[Put Away Line]]</calculatedColumnFormula>
@@ -5532,12 +5618,12 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="tbl_MaterialRequest" displayName="tbl_MaterialRequest" ref="A3:R18">
   <autoFilter ref="A3:R18" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}"/>
   <tableColumns count="18">
-    <tableColumn id="20" xr3:uid="{B9BDAC6D-879A-470A-ABB4-87ED00CCA6F0}" name="Request Number" totalsRowLabel="Total" dataDxfId="139" totalsRowDxfId="138"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Request Line" dataDxfId="137" totalsRowDxfId="136"/>
+    <tableColumn id="20" xr3:uid="{B9BDAC6D-879A-470A-ABB4-87ED00CCA6F0}" name="Request Number" totalsRowLabel="Total" dataDxfId="143" totalsRowDxfId="142"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Request Line" dataDxfId="141" totalsRowDxfId="140"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Request Date"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0600-00000A000000}" name="Required Date" dataDxfId="135" totalsRowDxfId="134"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0600-00000A000000}" name="Required Date" dataDxfId="139" totalsRowDxfId="138"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Requesting Department"/>
-    <tableColumn id="11" xr3:uid="{831BCE6C-DEE7-4065-962F-97D9A2507CC7}" name="Requester" dataDxfId="133" totalsRowDxfId="132"/>
+    <tableColumn id="11" xr3:uid="{831BCE6C-DEE7-4065-962F-97D9A2507CC7}" name="Requester" dataDxfId="137" totalsRowDxfId="136"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Material Code"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0600-000006000000}" name="Material Description"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0600-000007000000}" name="Base UoM">
@@ -5545,18 +5631,18 @@
     </tableColumn>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0600-000008000000}" name="Quantity Requested"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0600-000009000000}" name="Request Priority"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0600-00000D000000}" name="Available Stock (Ref)" dataDxfId="131">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0600-00000D000000}" name="Available Stock (Ref)" dataDxfId="135">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_MaterialRequest[[#This Row],[Material Code]],'10_Stock_Card'!F4:F32,'10_Stock_Card'!M4:M32,"",0,-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0600-00000E000000}" name="Stock Sufficiency Check" dataDxfId="130">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0600-00000E000000}" name="Stock Sufficiency Check" dataDxfId="134">
       <calculatedColumnFormula>IF(L4&gt;=J4,"Sufficient","Insufficient - Review")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{74FAE01D-9255-4B75-B167-77ECC7DC5BAF}" name="Approval Status" dataDxfId="129" totalsRowDxfId="128"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0600-00000C000000}" name="Total Issued (Ref)" dataDxfId="127" totalsRowDxfId="126">
+    <tableColumn id="18" xr3:uid="{74FAE01D-9255-4B75-B167-77ECC7DC5BAF}" name="Approval Status" dataDxfId="133" totalsRowDxfId="132"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0600-00000C000000}" name="Total Issued (Ref)" dataDxfId="131" totalsRowDxfId="130">
       <calculatedColumnFormula>IFERROR(_xlfn.XLOOKUP(tbl_MaterialRequest[[#This Row],[Request Line Key (Helper)]],tbl_GoodsIssue[MR],tbl_GoodsIssue[Quantity Issued]),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0600-00000F000000}" name="Request Status" dataDxfId="125" totalsRowDxfId="124"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0600-000010000000}" name="Remarks" dataDxfId="123" totalsRowDxfId="122"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0600-00000F000000}" name="Request Status" dataDxfId="129" totalsRowDxfId="128"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0600-000010000000}" name="Remarks" dataDxfId="127" totalsRowDxfId="126"/>
     <tableColumn id="17" xr3:uid="{00000000-0010-0000-0600-000011000000}" name="Request Line Key (Helper)" totalsRowFunction="count">
       <calculatedColumnFormula>tbl_MaterialRequest[[#This Row],[Request Number]]&amp;"-"&amp;tbl_MaterialRequest[[#This Row],[Request Line]]</calculatedColumnFormula>
     </tableColumn>
@@ -5577,35 +5663,35 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0700-000006000000}" name="Request Line Key (Helper)">
       <calculatedColumnFormula>tbl_PickingList[[#This Row],[Request Number]]&amp;"-"&amp;tbl_PickingList[[#This Row],[Request Line]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0700-000007000000}" name="Material Code" dataDxfId="121">
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0700-000007000000}" name="Material Code" dataDxfId="125">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PickingList[[#This Row],[Request Line Key (Helper)]],tbl_MaterialRequest[Request Line Key (Helper)],tbl_MaterialRequest[Material Code])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="Material Description" dataDxfId="120">
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0700-000008000000}" name="Material Description" dataDxfId="124">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PickingList[[#This Row],[Request Line Key (Helper)]],tbl_MaterialRequest[Request Line Key (Helper)],tbl_MaterialRequest[Material Description])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{C9E3CB77-E7C0-4337-8D57-40323596F0A3}" name="Base UoM" dataDxfId="119">
+    <tableColumn id="21" xr3:uid="{C9E3CB77-E7C0-4337-8D57-40323596F0A3}" name="Base UoM" dataDxfId="123">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PickingList[[#This Row],[Request Line Key (Helper)]],tbl_MaterialRequest[Request Line Key (Helper)],tbl_MaterialRequest[Base UoM])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="Requesting Department (Ref)" dataDxfId="118">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0700-000009000000}" name="Requesting Department (Ref)" dataDxfId="122">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PickingList[[#This Row],[Request Line Key (Helper)]],tbl_MaterialRequest[Request Line Key (Helper)],tbl_MaterialRequest[Requesting Department])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0700-00000A000000}" name="Request Priority (Ref)" dataDxfId="117">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0700-00000A000000}" name="Request Priority (Ref)" dataDxfId="121">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PickingList[[#This Row],[Request Line Key (Helper)]],tbl_MaterialRequest[Request Line Key (Helper)],tbl_MaterialRequest[Request Priority])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Quantity Requested (Ref)" dataDxfId="116">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0700-00000B000000}" name="Quantity Requested (Ref)" dataDxfId="120">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PickingList[[#This Row],[Request Line Key (Helper)]],tbl_MaterialRequest[Request Line Key (Helper)],tbl_MaterialRequest[Quantity Requested])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Pick Location " dataDxfId="115">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0700-00000C000000}" name="Pick Location " dataDxfId="119">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PickingList[[#This Row],[Material Code]],tbl_PutAway[Material Code],tbl_PutAway[To Location])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0700-00000E000000}" name="Available Stock" dataDxfId="114">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0700-00000E000000}" name="Available Stock" dataDxfId="118">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_PickingList[[#This Row],[Material Code]],'10_Stock_Card'!F4:F32,'10_Stock_Card'!M4:M32,"",0,-1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0700-000010000000}" name="Quantity Picked" dataDxfId="113"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0700-000011000000}" name="Pick Status" dataDxfId="112">
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0700-000010000000}" name="Quantity Picked" dataDxfId="117"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0700-000011000000}" name="Pick Status" dataDxfId="116">
       <calculatedColumnFormula>IF(tbl_PickingList[[#This Row],[Quantity Requested (Ref)]]=0,"Not Picked",IF(tbl_PickingList[[#This Row],[Quantity Picked]]&lt;tbl_PickingList[[#This Row],[Quantity Requested (Ref)]],"Partially Picked","Fully Picked"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="25" xr3:uid="{73D8D924-0876-4F34-9DBA-39EA7F81708E}" name="Picker" dataDxfId="111"/>
+    <tableColumn id="25" xr3:uid="{73D8D924-0876-4F34-9DBA-39EA7F81708E}" name="Picker" dataDxfId="115"/>
     <tableColumn id="19" xr3:uid="{00000000-0010-0000-0700-000013000000}" name="Remarks"/>
     <tableColumn id="20" xr3:uid="{00000000-0010-0000-0700-000014000000}" name="Pick Line Key (Helper)">
       <calculatedColumnFormula>tbl_PickingList[[#This Row],[Pick Number]]&amp;"-"&amp;tbl_PickingList[[#This Row],[Pick Line]]</calculatedColumnFormula>
@@ -5624,13 +5710,13 @@
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0800-000003000000}" name="GI Date"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0800-000004000000}" name="Pick Number"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0800-000005000000}" name="Pick Line"/>
-    <tableColumn id="19" xr3:uid="{E93C14AF-94CF-4F14-81CC-82A7578004AD}" name="Request Number" dataDxfId="110">
+    <tableColumn id="19" xr3:uid="{E93C14AF-94CF-4F14-81CC-82A7578004AD}" name="Request Number" dataDxfId="114">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_GoodsIssue[[#This Row],[Pick Line Key (Helper)]],tbl_PickingList[Pick Line Key (Helper)],tbl_PickingList[Request Number])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="20" xr3:uid="{38A75A8A-6A06-4489-86DF-2EE0CE3971EF}" name="Request Line" dataDxfId="109">
+    <tableColumn id="20" xr3:uid="{38A75A8A-6A06-4489-86DF-2EE0CE3971EF}" name="Request Line" dataDxfId="113">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_GoodsIssue[[#This Row],[Pick Line Key (Helper)]],tbl_PickingList[Pick Line Key (Helper)],tbl_PickingList[Request Line])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="Pick Line Key (Helper)" dataDxfId="108">
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0800-000006000000}" name="Pick Line Key (Helper)" dataDxfId="112">
       <calculatedColumnFormula>D4&amp;"-"&amp;E4</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0800-000007000000}" name="Material Code">
@@ -5639,32 +5725,32 @@
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0800-000008000000}" name="Material Description">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_GoodsIssue[[#This Row],[Material Code]],tbl_MasterMaterial[Material Code],tbl_MasterMaterial[Material Description])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0800-000009000000}" name="Base UoM" dataDxfId="107">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0800-000009000000}" name="Base UoM" dataDxfId="111">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_GoodsIssue[[#This Row],[Material Code]],tbl_MasterMaterial[Material Code],tbl_MasterMaterial[Base UoM])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0800-00000A000000}" name="Issuing Location (Ref)" dataDxfId="106">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0800-00000A000000}" name="Issuing Location (Ref)" dataDxfId="110">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_GoodsIssue[[#This Row],[Pick Line Key (Helper)]],tbl_PickingList[Pick Line Key (Helper)],tbl_PickingList[[Pick Location ]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0800-00000B000000}" name="Requesting Department (Ref)" dataDxfId="105">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0800-00000B000000}" name="Requesting Department (Ref)" dataDxfId="109">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_GoodsIssue[[#This Row],[Pick Line Key (Helper)]],tbl_PickingList[Pick Line Key (Helper)],tbl_PickingList[Requesting Department (Ref)])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0800-00000C000000}" name="Quantity Picked (Ref)" dataDxfId="104">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0800-00000C000000}" name="Quantity Picked (Ref)" dataDxfId="108">
       <calculatedColumnFormula>_xlfn.XLOOKUP(tbl_GoodsIssue[[#This Row],[Pick Line Key (Helper)]],tbl_PickingList[Pick Line Key (Helper)],tbl_PickingList[Quantity Picked])</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0800-00000D000000}" name="Quantity Issued"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0800-00000E000000}" name="Issue Variance" dataDxfId="103">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0800-00000E000000}" name="Issue Variance" dataDxfId="107">
       <calculatedColumnFormula>tbl_GoodsIssue[[#This Row],[Quantity Issued]]-tbl_GoodsIssue[[#This Row],[Quantity Picked (Ref)]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{604A2A6F-C4DD-4034-9B7B-D193996479E5}" name="Issue Status" dataDxfId="102">
+    <tableColumn id="15" xr3:uid="{604A2A6F-C4DD-4034-9B7B-D193996479E5}" name="Issue Status" dataDxfId="106">
       <calculatedColumnFormula>IF(tbl_GoodsIssue[[#This Row],[Quantity Issued]]&lt;tbl_GoodsIssue[[#This Row],[Quantity Picked (Ref)]],"Partial","Completed")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{90D76B52-520C-4D83-81A3-B6E72FB0F149}" name="Issued By" dataDxfId="101"/>
-    <tableColumn id="22" xr3:uid="{76096732-D4A3-4A12-8DD0-430477B5B0BF}" name="Received By" dataDxfId="100"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0800-000010000000}" name="Remarks" dataDxfId="99"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0800-000011000000}" name="GI Line Key (Helper)" dataDxfId="98">
+    <tableColumn id="21" xr3:uid="{90D76B52-520C-4D83-81A3-B6E72FB0F149}" name="Issued By" dataDxfId="105"/>
+    <tableColumn id="22" xr3:uid="{76096732-D4A3-4A12-8DD0-430477B5B0BF}" name="Received By" dataDxfId="104"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0800-000010000000}" name="Remarks" dataDxfId="103"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0800-000011000000}" name="GI Line Key (Helper)" dataDxfId="102">
       <calculatedColumnFormula>tbl_GoodsIssue[[#This Row],[GI Number]]&amp;"-"&amp;tbl_GoodsIssue[[#This Row],[GI Line]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{21F1F36F-2396-482F-BFCE-12F60C905BC9}" name="MR" dataDxfId="97">
+    <tableColumn id="23" xr3:uid="{21F1F36F-2396-482F-BFCE-12F60C905BC9}" name="MR" dataDxfId="101">
       <calculatedColumnFormula>tbl_GoodsIssue[[#This Row],[Request Number]]&amp;"-"&amp;tbl_GoodsIssue[[#This Row],[Request Line]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6014,10 +6100,10 @@
         <v>24</v>
       </c>
       <c r="K5" s="3">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="L5" s="3">
-        <v>50</v>
+        <v>85</v>
       </c>
       <c r="M5" s="3">
         <v>21</v>
@@ -6059,10 +6145,10 @@
         <v>19</v>
       </c>
       <c r="K6" s="3">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="L6" s="3">
-        <v>300</v>
+        <v>140</v>
       </c>
       <c r="M6" s="3">
         <v>7</v>
@@ -6149,7 +6235,7 @@
         <v>35</v>
       </c>
       <c r="K8" s="3">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="L8" s="3">
         <v>200</v>
@@ -6284,10 +6370,10 @@
         <v>19</v>
       </c>
       <c r="K11" s="3">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="L11" s="3">
-        <v>80</v>
+        <v>125</v>
       </c>
       <c r="M11" s="3">
         <v>12</v>
@@ -6419,10 +6505,10 @@
         <v>24</v>
       </c>
       <c r="K14" s="3">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="L14" s="3">
-        <v>10</v>
+        <v>125</v>
       </c>
       <c r="M14" s="3">
         <v>45</v>
@@ -6464,7 +6550,7 @@
         <v>24</v>
       </c>
       <c r="K15" s="3">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="L15" s="3">
         <v>120</v>
@@ -6599,7 +6685,7 @@
         <v>24</v>
       </c>
       <c r="K18" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="L18" s="3">
         <v>50</v>
@@ -6644,7 +6730,7 @@
         <v>19</v>
       </c>
       <c r="K19" s="3">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="L19" s="3">
         <v>200</v>
@@ -6689,10 +6775,10 @@
         <v>24</v>
       </c>
       <c r="K20" s="3">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="L20" s="3">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="M20" s="3">
         <v>25</v>
@@ -6779,10 +6865,10 @@
         <v>19</v>
       </c>
       <c r="K22" s="3">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="L22" s="3">
-        <v>400</v>
+        <v>250</v>
       </c>
       <c r="M22" s="3">
         <v>9</v>
@@ -6824,10 +6910,10 @@
         <v>24</v>
       </c>
       <c r="K23" s="3">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="L23" s="3">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="M23" s="3">
         <v>40</v>
@@ -6863,35 +6949,43 @@
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <conditionalFormatting sqref="A31:E53">
-    <cfRule type="expression" dxfId="82" priority="103">
+    <cfRule type="expression" dxfId="86" priority="105">
       <formula>$E31="Inactive"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="81" priority="104">
+    <cfRule type="expression" dxfId="85" priority="106">
       <formula>#REF!="Critical Spare"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A4:O23">
-    <cfRule type="expression" dxfId="80" priority="28">
+  <conditionalFormatting sqref="A4:J23 M4:O23">
+    <cfRule type="expression" dxfId="84" priority="30">
       <formula>$N4="Inactive"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="79" priority="29">
+    <cfRule type="expression" dxfId="83" priority="31">
       <formula>$I4="Critical Spare"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A24:O30 A54:O498">
-    <cfRule type="expression" dxfId="78" priority="20">
+    <cfRule type="expression" dxfId="82" priority="22">
       <formula>$O24="Inactive"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="77" priority="21">
+    <cfRule type="expression" dxfId="81" priority="23">
       <formula>$I24="Critical Spare"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F4:F23">
-    <cfRule type="duplicateValues" dxfId="76" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H23">
-    <cfRule type="containsText" dxfId="75" priority="1" operator="containsText" text="A">
+    <cfRule type="containsText" dxfId="79" priority="3" operator="containsText" text="A">
       <formula>NOT(ISERROR(SEARCH("A",H4)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K4:L23">
+    <cfRule type="expression" dxfId="3" priority="1">
+      <formula>$N4="Inactive"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="2">
+      <formula>$I4="Critical Spare"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="8">
@@ -8908,33 +9002,33 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="A33:A39 A41:A518">
-    <cfRule type="expression" dxfId="18" priority="2">
+    <cfRule type="expression" dxfId="22" priority="2">
       <formula>$A33="Receipt"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="3">
+    <cfRule type="expression" dxfId="21" priority="3">
       <formula>$A33="Issue"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4:B32">
-    <cfRule type="expression" dxfId="16" priority="5">
+    <cfRule type="expression" dxfId="20" priority="5">
       <formula>$B4="Goods Receipt"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="6">
+    <cfRule type="expression" dxfId="19" priority="6">
       <formula>$B4="Goods Issue"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L4:L32">
-    <cfRule type="expression" dxfId="14" priority="1">
+    <cfRule type="expression" dxfId="18" priority="1">
       <formula>$L4&lt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L33:L518">
-    <cfRule type="expression" dxfId="13" priority="4">
+    <cfRule type="expression" dxfId="17" priority="4">
       <formula>$L33&lt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M4:M32">
-    <cfRule type="expression" dxfId="12" priority="7">
+    <cfRule type="expression" dxfId="16" priority="7">
       <formula>$M4&lt;0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9646,50 +9740,50 @@
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <conditionalFormatting sqref="A24:A47">
-    <cfRule type="expression" dxfId="11" priority="117">
+    <cfRule type="expression" dxfId="15" priority="117">
       <formula>#REF!="Shortage"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="118">
+    <cfRule type="expression" dxfId="14" priority="118">
       <formula>#REF!="Overage"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="119">
+    <cfRule type="expression" dxfId="13" priority="119">
       <formula>#REF!="Match"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C24:D47">
-    <cfRule type="expression" dxfId="8" priority="121">
+    <cfRule type="expression" dxfId="12" priority="121">
       <formula>$C24="Under Investigation"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M12:O23 M48:O504">
-    <cfRule type="expression" dxfId="7" priority="3">
+    <cfRule type="expression" dxfId="11" priority="3">
       <formula>$M12="Shortage"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="4">
+    <cfRule type="expression" dxfId="10" priority="4">
       <formula>$M12="Overage"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="5">
+    <cfRule type="expression" dxfId="9" priority="5">
       <formula>$M12="Match"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N4:P11">
-    <cfRule type="expression" dxfId="4" priority="110">
+    <cfRule type="expression" dxfId="8" priority="110">
       <formula>$N4="Shortage"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="111">
+    <cfRule type="expression" dxfId="7" priority="111">
       <formula>$N4="Overage"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="112">
+    <cfRule type="expression" dxfId="6" priority="112">
       <formula>$N4="Match"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q12:R23 Q48:R504">
-    <cfRule type="expression" dxfId="1" priority="6">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>$Q12="Under Investigation"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R4:R11 T4:T11">
-    <cfRule type="expression" dxfId="0" priority="113">
+    <cfRule type="expression" dxfId="4" priority="113">
       <formula>$R4="Under Investigation"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10248,15 +10342,15 @@
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <conditionalFormatting sqref="A4:I13">
-    <cfRule type="expression" dxfId="74" priority="37">
+    <cfRule type="expression" dxfId="78" priority="37">
       <formula>$I4="Inactive"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="73" priority="38">
+    <cfRule type="expression" dxfId="77" priority="38">
       <formula>$H4="Preferred"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H14:H21">
-    <cfRule type="expression" dxfId="72" priority="7">
+    <cfRule type="expression" dxfId="76" priority="7">
       <formula>$H14="Under Review"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11202,36 +11296,36 @@
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <conditionalFormatting sqref="A29:G36 A46:B55 A56:G512">
-    <cfRule type="expression" dxfId="71" priority="2">
+    <cfRule type="expression" dxfId="75" priority="2">
       <formula>$G29="Inactive"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="70" priority="3">
+    <cfRule type="expression" dxfId="74" priority="3">
       <formula>$D29="Hazardous"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A4:H15 A16:F17 H16:H17 A18:H28">
-    <cfRule type="expression" dxfId="69" priority="41">
+    <cfRule type="expression" dxfId="73" priority="41">
       <formula>$H4="Inactive"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="68" priority="42">
+    <cfRule type="expression" dxfId="72" priority="42">
       <formula>$E4="Hazardous"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E29:E36 E56:E512">
-    <cfRule type="expression" dxfId="67" priority="4">
+    <cfRule type="expression" dxfId="71" priority="4">
       <formula>$E29="No"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F4:F28">
-    <cfRule type="expression" dxfId="66" priority="46">
+    <cfRule type="expression" dxfId="70" priority="46">
       <formula>$F4="No"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G16">
-    <cfRule type="expression" dxfId="65" priority="105">
+    <cfRule type="expression" dxfId="69" priority="105">
       <formula>$H17="Inactive"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="64" priority="106">
+    <cfRule type="expression" dxfId="68" priority="106">
       <formula>$E17="Hazardous"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13102,53 +13196,53 @@
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <conditionalFormatting sqref="C33:C79">
-    <cfRule type="expression" dxfId="63" priority="127">
+    <cfRule type="expression" dxfId="67" priority="127">
       <formula>$C33="Urgent"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G33:G79">
-    <cfRule type="expression" dxfId="62" priority="131">
+    <cfRule type="expression" dxfId="66" priority="131">
       <formula>$G33="Cancelled"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="61" priority="132">
+    <cfRule type="expression" dxfId="65" priority="132">
       <formula>$G33="Closed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="60" priority="133">
+    <cfRule type="expression" dxfId="64" priority="133">
       <formula>$G33="Open"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L4:L26 L28:L29">
-    <cfRule type="expression" dxfId="59" priority="56">
+    <cfRule type="expression" dxfId="63" priority="56">
       <formula>$L4="Urgent"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N30:N32 N80:N515">
-    <cfRule type="expression" dxfId="58" priority="3">
+    <cfRule type="expression" dxfId="62" priority="3">
       <formula>$N30="Urgent"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q4:Q26 Q28:Q29">
-    <cfRule type="expression" dxfId="57" priority="1">
+    <cfRule type="expression" dxfId="61" priority="1">
       <formula>$Q4="Partial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="56" priority="64">
+    <cfRule type="expression" dxfId="60" priority="64">
       <formula>$Q4="Cancelled"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="55" priority="65">
+    <cfRule type="expression" dxfId="59" priority="65">
       <formula>$Q4="Closed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="54" priority="66">
+    <cfRule type="expression" dxfId="58" priority="66">
       <formula>$Q4="Open"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R30:R32 R80:R515">
-    <cfRule type="expression" dxfId="53" priority="4">
+    <cfRule type="expression" dxfId="57" priority="4">
       <formula>$R30="Cancelled"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="52" priority="5">
+    <cfRule type="expression" dxfId="56" priority="5">
       <formula>$R30="Closed"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="51" priority="6">
+    <cfRule type="expression" dxfId="55" priority="6">
       <formula>$R30="Open"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15383,31 +15477,31 @@
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <conditionalFormatting sqref="K24:K35">
-    <cfRule type="expression" dxfId="50" priority="124">
+    <cfRule type="expression" dxfId="54" priority="124">
       <formula>$K24="Fully Rejected"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="49" priority="125">
+    <cfRule type="expression" dxfId="53" priority="125">
       <formula>$K24="Partially Accepted"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S22:S23 S36:S512">
-    <cfRule type="expression" dxfId="48" priority="6">
+    <cfRule type="expression" dxfId="52" priority="6">
       <formula>$S22="Fully Rejected"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="47" priority="7">
+    <cfRule type="expression" dxfId="51" priority="7">
       <formula>$S22="Partially Accepted"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U4:U21">
-    <cfRule type="expression" dxfId="46" priority="61">
+    <cfRule type="expression" dxfId="50" priority="61">
       <formula>$U4="Fully Rejected"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="45" priority="62">
+    <cfRule type="expression" dxfId="49" priority="62">
       <formula>$U4="Partially Accepted"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z4:Z21">
-    <cfRule type="expression" dxfId="44" priority="1">
+    <cfRule type="expression" dxfId="48" priority="1">
       <formula>$Z4="Late"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17236,26 +17330,26 @@
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <conditionalFormatting sqref="Q22:Q513">
-    <cfRule type="expression" dxfId="43" priority="5">
+    <cfRule type="expression" dxfId="47" priority="5">
       <formula>$Q22="Mismatch - Review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R4:R20">
-    <cfRule type="duplicateValues" dxfId="42" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="T4:T20">
-    <cfRule type="expression" dxfId="41" priority="2">
+    <cfRule type="expression" dxfId="45" priority="2">
       <formula>$T4="Mismatch - Review"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U4:U20">
-    <cfRule type="expression" dxfId="40" priority="3">
+    <cfRule type="expression" dxfId="44" priority="3">
       <formula>$U4="Partial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="39" priority="74">
+    <cfRule type="expression" dxfId="43" priority="74">
       <formula>$U4="Exception - Needs Review"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="75">
+    <cfRule type="expression" dxfId="42" priority="75">
       <formula>$U4="Completed"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -18338,28 +18432,28 @@
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <conditionalFormatting sqref="I19:I507">
-    <cfRule type="expression" dxfId="37" priority="2">
+    <cfRule type="expression" dxfId="41" priority="2">
       <formula>$I19="Urgent"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K4:K18">
-    <cfRule type="expression" dxfId="36" priority="83">
+    <cfRule type="expression" dxfId="40" priority="83">
       <formula>$K4="Urgent"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M4:N18">
-    <cfRule type="expression" dxfId="35" priority="80">
+    <cfRule type="expression" dxfId="39" priority="80">
       <formula>$M4="Insufficient - Review"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="34" priority="81">
+    <cfRule type="expression" dxfId="38" priority="81">
       <formula>$M4="Sufficient"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N19:N507">
-    <cfRule type="expression" dxfId="33" priority="3">
+    <cfRule type="expression" dxfId="37" priority="3">
       <formula>$N19="Insufficient - Review"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="32" priority="4">
+    <cfRule type="expression" dxfId="36" priority="4">
       <formula>$N19="Sufficient"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19361,31 +19455,31 @@
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <conditionalFormatting sqref="K4:K18 K80:K507">
-    <cfRule type="expression" dxfId="31" priority="2">
+    <cfRule type="expression" dxfId="35" priority="2">
       <formula>$K4="Urgent"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P4:P15">
-    <cfRule type="expression" dxfId="30" priority="88">
+    <cfRule type="expression" dxfId="34" priority="88">
       <formula>$P4="Fully Picked"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P4:Q15">
-    <cfRule type="expression" dxfId="29" priority="87">
+    <cfRule type="expression" dxfId="33" priority="87">
       <formula>$P4="Partially Picked"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="28" priority="89">
+    <cfRule type="expression" dxfId="32" priority="89">
       <formula>$P4="Not Picked"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q16:Q17 Q80:Q507">
-    <cfRule type="expression" dxfId="27" priority="4">
+    <cfRule type="expression" dxfId="31" priority="4">
       <formula>$Q16="Partially Picked"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="5">
+    <cfRule type="expression" dxfId="30" priority="5">
       <formula>$Q16="Fully Picked"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="25" priority="6">
+    <cfRule type="expression" dxfId="29" priority="6">
       <formula>$Q16="Not Picked"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -20687,32 +20781,32 @@
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <conditionalFormatting sqref="P4:Q15">
-    <cfRule type="expression" dxfId="24" priority="92">
+    <cfRule type="expression" dxfId="28" priority="92">
       <formula>$P4&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q4:Q15">
-    <cfRule type="expression" dxfId="23" priority="1">
+    <cfRule type="expression" dxfId="27" priority="1">
       <formula>$Q4="Completed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q4:S15">
-    <cfRule type="expression" dxfId="22" priority="95">
+    <cfRule type="expression" dxfId="26" priority="95">
       <formula>#REF!&lt;&gt;"N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q16:S16 O17:Q28 Q29:S507">
-    <cfRule type="expression" dxfId="21" priority="96">
+    <cfRule type="expression" dxfId="25" priority="96">
       <formula>#REF!&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R17:R28">
-    <cfRule type="expression" dxfId="20" priority="100">
+    <cfRule type="expression" dxfId="24" priority="100">
       <formula>$R17&lt;&gt;"N/A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T16:U16 T29:U507">
-    <cfRule type="expression" dxfId="19" priority="4">
+    <cfRule type="expression" dxfId="23" priority="4">
       <formula>$T16&lt;&gt;"N/A"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>